<commit_message>
Updated NGA_grids_kan model - 2025-12-06 12:52
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{796AA07D-9482-48BE-8953-108D7CE18CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{983FE04C-7E82-40F9-8D9D-4D23735A4138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1997,7 +1997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125D380C-FADE-48A0-B86F-D055680B235D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC8C85DE-BCA1-4CD8-A98B-53F271DC9606}">
   <dimension ref="B9:E145"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NGA_grids_kan model - 2025-12-11 11:00
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E775D7D-5B59-4599-9746-E4659EF2481F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A920A3C-E183-4B64-8D3B-AC017FBAFC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1997,7 +1997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A49DE6E-3AD1-46DC-8E7C-FCB76B64A541}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34B4A914-AA38-4E24-9706-5C632F7DB4F8}">
   <dimension ref="B9:E145"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>